<commit_message>
Update: GTR View 3
</commit_message>
<xml_diff>
--- a/docker/postgres/users-seed/users-seed.xlsx
+++ b/docker/postgres/users-seed/users-seed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edinson\Documents\SpringBoot\ALBRUGROUP\docker\postgres\users-seed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2ACFE5-443A-426B-8E67-737E3032BC4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC6408B-5C8D-42E4-B91F-817F4BA0B4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="2475" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="15585" yWindow="2985" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="users-seed" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="296">
   <si>
     <t>empleado_id</t>
   </si>
@@ -916,6 +916,18 @@
   </si>
   <si>
     <t>Av Demo 1051</t>
+  </si>
+  <si>
+    <t>Q8%9gPh$Sr</t>
+  </si>
+  <si>
+    <t>PASSWORD</t>
+  </si>
+  <si>
+    <t>LZaYJfXtVK</t>
+  </si>
+  <si>
+    <t>y_qgqWsDSV</t>
   </si>
 </sst>
 </file>
@@ -925,10 +937,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -951,10 +971,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -969,17 +990,24 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="16">
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
@@ -1021,13 +1049,10 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1044,8 +1069,8 @@
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatosExternos_1" connectionId="1" xr16:uid="{D2EE246D-06EF-4D2E-A245-9E0EBF54F313}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="20">
-    <queryTableFields count="19">
+  <queryTableRefresh nextId="21" unboundColumnsRight="1">
+    <queryTableFields count="20">
       <queryTableField id="1" name="empleado_id" tableColumnId="1"/>
       <queryTableField id="2" name="usuario_id" tableColumnId="2"/>
       <queryTableField id="3" name="contrato_id" tableColumnId="3"/>
@@ -1065,34 +1090,53 @@
       <queryTableField id="17" name="hora_salida" tableColumnId="17"/>
       <queryTableField id="18" name="inicio_almuerzo" tableColumnId="18"/>
       <queryTableField id="19" name="fin_almuerzo" tableColumnId="19"/>
+      <queryTableField id="20" dataBound="0" tableColumnId="20"/>
     </queryTableFields>
   </queryTableRefresh>
 </queryTable>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{64F05A49-00C3-4190-AFA5-1C9AC74EA2CE}" name="users_seed" displayName="users_seed" ref="A1:S52" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:S52" xr:uid="{64F05A49-00C3-4190-AFA5-1C9AC74EA2CE}"/>
-  <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{945557A6-9D57-4DB1-92F9-EC6350595D37}" uniqueName="1" name="empleado_id" queryTableFieldId="1" dataDxfId="13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{64F05A49-00C3-4190-AFA5-1C9AC74EA2CE}" name="users_seed" displayName="users_seed" ref="A1:T52" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:T52" xr:uid="{64F05A49-00C3-4190-AFA5-1C9AC74EA2CE}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="ADMINISTRADOR"/>
+        <filter val="ASESOR_BACKOFFICE"/>
+        <filter val="ASESOR_GTR"/>
+        <filter val="ASESOR_VENTAS"/>
+        <filter val="COMMUNITY"/>
+        <filter val="RRHH"/>
+        <filter val="SUPERVISOR_VENTAS"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="15">
+      <filters>
+        <filter val="16:00:00"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="20">
+    <tableColumn id="1" xr3:uid="{945557A6-9D57-4DB1-92F9-EC6350595D37}" uniqueName="1" name="empleado_id" queryTableFieldId="1" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{7A1088D5-AA0D-4D8F-BC77-5BFDEE8F7170}" uniqueName="2" name="usuario_id" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{CCEEF7F6-4F47-45F9-AEC4-814A362E9AA1}" uniqueName="3" name="contrato_id" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{83AB7252-C401-4208-8C65-22BE47EEDCBB}" uniqueName="4" name="horario_id" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{74D8849A-7BB1-4490-9EC7-34E2E2BF1D1E}" uniqueName="5" name="nombres" queryTableFieldId="5" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{ECA68842-1FE3-4ADC-A73C-BF2948A95E80}" uniqueName="6" name="apellidos" queryTableFieldId="6" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{CAFC01E5-AFF3-49B6-B20F-A3710218E73C}" uniqueName="7" name="puesto_trabajo" queryTableFieldId="7" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{7518104A-000F-4ABD-921B-608A103DDFE5}" uniqueName="8" name="numero_documento" queryTableFieldId="8" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{7D0045CC-BF36-4407-833C-4769D389D038}" uniqueName="9" name="correo_personal" queryTableFieldId="9" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{B4445341-B733-42A4-9DAA-7F38F8C53CF3}" uniqueName="10" name="username" queryTableFieldId="10" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{70795878-C198-4257-8559-7EA937BE0F5C}" uniqueName="11" name="celular_personal" queryTableFieldId="11" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{9BBA232E-754D-43C6-89BD-FB2CCB9EE50A}" uniqueName="12" name="fecha_nacimiento" queryTableFieldId="12" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{D165E82A-0565-4D2A-A2C1-9A20141CC2A4}" uniqueName="13" name="direccion" queryTableFieldId="13" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{E412DF89-6243-423A-8977-A1521C419C75}" uniqueName="14" name="cuenta_bancaria" queryTableFieldId="14" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{1C95BD7B-82C7-4617-9587-E6C510EF7125}" uniqueName="15" name="cuenta_interbancaria" queryTableFieldId="15" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{76CF0A87-B350-4EBF-A806-D5D66507ECE2}" uniqueName="16" name="hora_entrada" queryTableFieldId="16" dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{80484A11-AB11-45BD-BBAA-153B35B43755}" uniqueName="17" name="hora_salida" queryTableFieldId="17" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{74D8849A-7BB1-4490-9EC7-34E2E2BF1D1E}" uniqueName="5" name="nombres" queryTableFieldId="5" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{ECA68842-1FE3-4ADC-A73C-BF2948A95E80}" uniqueName="6" name="apellidos" queryTableFieldId="6" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{CAFC01E5-AFF3-49B6-B20F-A3710218E73C}" uniqueName="7" name="puesto_trabajo" queryTableFieldId="7" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{7518104A-000F-4ABD-921B-608A103DDFE5}" uniqueName="8" name="numero_documento" queryTableFieldId="8" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{7D0045CC-BF36-4407-833C-4769D389D038}" uniqueName="9" name="correo_personal" queryTableFieldId="9" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{B4445341-B733-42A4-9DAA-7F38F8C53CF3}" uniqueName="10" name="username" queryTableFieldId="10" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{70795878-C198-4257-8559-7EA937BE0F5C}" uniqueName="11" name="celular_personal" queryTableFieldId="11" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{9BBA232E-754D-43C6-89BD-FB2CCB9EE50A}" uniqueName="12" name="fecha_nacimiento" queryTableFieldId="12" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{D165E82A-0565-4D2A-A2C1-9A20141CC2A4}" uniqueName="13" name="direccion" queryTableFieldId="13" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{E412DF89-6243-423A-8977-A1521C419C75}" uniqueName="14" name="cuenta_bancaria" queryTableFieldId="14" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{1C95BD7B-82C7-4617-9587-E6C510EF7125}" uniqueName="15" name="cuenta_interbancaria" queryTableFieldId="15" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{76CF0A87-B350-4EBF-A806-D5D66507ECE2}" uniqueName="16" name="hora_entrada" queryTableFieldId="16" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{80484A11-AB11-45BD-BBAA-153B35B43755}" uniqueName="17" name="hora_salida" queryTableFieldId="17" dataDxfId="2"/>
     <tableColumn id="18" xr3:uid="{56983649-142C-458B-A787-8803EF5C42C6}" uniqueName="18" name="inicio_almuerzo" queryTableFieldId="18" dataDxfId="1"/>
-    <tableColumn id="19" xr3:uid="{137EC0B4-9881-47BC-9A91-35198F7493DB}" uniqueName="19" name="fin_almuerzo" queryTableFieldId="19" dataDxfId="14"/>
+    <tableColumn id="19" xr3:uid="{137EC0B4-9881-47BC-9A91-35198F7493DB}" uniqueName="19" name="fin_almuerzo" queryTableFieldId="19" dataDxfId="0"/>
+    <tableColumn id="20" xr3:uid="{2F07A5DA-72AF-4D8E-BBA3-9BDCEB7E6C1C}" uniqueName="20" name="PASSWORD" queryTableFieldId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1361,10 +1405,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F5ACDB5-8359-4986-95E9-473CA3E4D90E}">
-  <dimension ref="A1:S52"/>
+  <dimension ref="A1:T55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15" style="2" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="13.42578125" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="12.42578125" hidden="1" customWidth="1"/>
@@ -1383,9 +1427,10 @@
     <col min="17" max="17" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.42578125" hidden="1" customWidth="1"/>
     <col min="19" max="19" width="15" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1443,8 +1488,11 @@
       <c r="S1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T1" s="2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1001</v>
       </c>
@@ -1502,8 +1550,9 @@
       <c r="S2" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T2"/>
+    </row>
+    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1002</v>
       </c>
@@ -1562,7 +1611,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>1003</v>
       </c>
@@ -1620,8 +1669,9 @@
       <c r="S4" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T4"/>
+    </row>
+    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>1004</v>
       </c>
@@ -1679,8 +1729,9 @@
       <c r="S5" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T5"/>
+    </row>
+    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>1005</v>
       </c>
@@ -1739,7 +1790,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>1006</v>
       </c>
@@ -1797,8 +1848,9 @@
       <c r="S7" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T7"/>
+    </row>
+    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>1007</v>
       </c>
@@ -1856,8 +1908,9 @@
       <c r="S8" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T8"/>
+    </row>
+    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>1008</v>
       </c>
@@ -1915,8 +1968,9 @@
       <c r="S9" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T9"/>
+    </row>
+    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>1009</v>
       </c>
@@ -1974,8 +2028,9 @@
       <c r="S10" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T10"/>
+    </row>
+    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>1010</v>
       </c>
@@ -2033,8 +2088,9 @@
       <c r="S11" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T11"/>
+    </row>
+    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>1011</v>
       </c>
@@ -2092,8 +2148,9 @@
       <c r="S12" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T12"/>
+    </row>
+    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>1012</v>
       </c>
@@ -2151,8 +2208,9 @@
       <c r="S13" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T13"/>
+    </row>
+    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>1013</v>
       </c>
@@ -2210,8 +2268,9 @@
       <c r="S14" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T14"/>
+    </row>
+    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>1014</v>
       </c>
@@ -2269,8 +2328,9 @@
       <c r="S15" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T15"/>
+    </row>
+    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>1015</v>
       </c>
@@ -2328,8 +2388,9 @@
       <c r="S16" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T16"/>
+    </row>
+    <row r="17" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>1016</v>
       </c>
@@ -2387,8 +2448,9 @@
       <c r="S17" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T17"/>
+    </row>
+    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>1017</v>
       </c>
@@ -2446,8 +2508,9 @@
       <c r="S18" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T18"/>
+    </row>
+    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>1018</v>
       </c>
@@ -2505,8 +2568,9 @@
       <c r="S19" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T19"/>
+    </row>
+    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>1019</v>
       </c>
@@ -2564,8 +2628,9 @@
       <c r="S20" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T20"/>
+    </row>
+    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>1020</v>
       </c>
@@ -2624,7 +2689,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>1021</v>
       </c>
@@ -2682,8 +2747,9 @@
       <c r="S22" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T22"/>
+    </row>
+    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>1022</v>
       </c>
@@ -2741,8 +2807,9 @@
       <c r="S23" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T23"/>
+    </row>
+    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>1023</v>
       </c>
@@ -2800,8 +2867,9 @@
       <c r="S24" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T24"/>
+    </row>
+    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>1024</v>
       </c>
@@ -2859,8 +2927,9 @@
       <c r="S25" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T25"/>
+    </row>
+    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>1025</v>
       </c>
@@ -2918,8 +2987,9 @@
       <c r="S26" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T26"/>
+    </row>
+    <row r="27" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>1026</v>
       </c>
@@ -2977,8 +3047,11 @@
       <c r="S27" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T27" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>1027</v>
       </c>
@@ -3036,8 +3109,9 @@
       <c r="S28" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T28"/>
+    </row>
+    <row r="29" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>1028</v>
       </c>
@@ -3095,8 +3169,9 @@
       <c r="S29" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T29"/>
+    </row>
+    <row r="30" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>1029</v>
       </c>
@@ -3154,8 +3229,11 @@
       <c r="S30" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T30" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>1030</v>
       </c>
@@ -3213,8 +3291,9 @@
       <c r="S31" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T31"/>
+    </row>
+    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>1031</v>
       </c>
@@ -3272,8 +3351,9 @@
       <c r="S32" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T32"/>
+    </row>
+    <row r="33" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>1032</v>
       </c>
@@ -3331,8 +3411,9 @@
       <c r="S33" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T33"/>
+    </row>
+    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>1033</v>
       </c>
@@ -3390,8 +3471,9 @@
       <c r="S34" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T34"/>
+    </row>
+    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>1034</v>
       </c>
@@ -3449,8 +3531,9 @@
       <c r="S35" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T35"/>
+    </row>
+    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>1035</v>
       </c>
@@ -3509,7 +3592,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>1036</v>
       </c>
@@ -3567,8 +3650,9 @@
       <c r="S37" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T37"/>
+    </row>
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>1037</v>
       </c>
@@ -3626,8 +3710,9 @@
       <c r="S38" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T38"/>
+    </row>
+    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>1038</v>
       </c>
@@ -3685,8 +3770,9 @@
       <c r="S39" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T39"/>
+    </row>
+    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>1039</v>
       </c>
@@ -3744,8 +3830,9 @@
       <c r="S40" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T40"/>
+    </row>
+    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>1040</v>
       </c>
@@ -3803,8 +3890,9 @@
       <c r="S41" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T41"/>
+    </row>
+    <row r="42" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>1041</v>
       </c>
@@ -3832,7 +3920,7 @@
       <c r="I42" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="J42" s="3" t="s">
+      <c r="J42" s="6" t="s">
         <v>237</v>
       </c>
       <c r="K42" s="2">
@@ -3862,8 +3950,11 @@
       <c r="S42" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T42" s="2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>1042</v>
       </c>
@@ -3921,8 +4012,11 @@
       <c r="S43" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T43" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>1043</v>
       </c>
@@ -3980,8 +4074,9 @@
       <c r="S44" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T44"/>
+    </row>
+    <row r="45" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>1044</v>
       </c>
@@ -4039,8 +4134,9 @@
       <c r="S45" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T45"/>
+    </row>
+    <row r="46" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>1045</v>
       </c>
@@ -4098,8 +4194,9 @@
       <c r="S46" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T46"/>
+    </row>
+    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>1046</v>
       </c>
@@ -4157,8 +4254,9 @@
       <c r="S47" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T47"/>
+    </row>
+    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>1047</v>
       </c>
@@ -4216,8 +4314,9 @@
       <c r="S48" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T48"/>
+    </row>
+    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>1048</v>
       </c>
@@ -4275,8 +4374,9 @@
       <c r="S49" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T49"/>
+    </row>
+    <row r="50" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>1049</v>
       </c>
@@ -4334,8 +4434,9 @@
       <c r="S50" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T50"/>
+    </row>
+    <row r="51" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>1050</v>
       </c>
@@ -4393,8 +4494,9 @@
       <c r="S51" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T51"/>
+    </row>
+    <row r="52" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>1051</v>
       </c>
@@ -4452,11 +4554,18 @@
       <c r="S52" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="T52"/>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="T55"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J42" r:id="rId1" xr:uid="{11A69FDB-E49E-44F4-9FD1-55C6F553F529}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update: Correcion 1 Schdule
</commit_message>
<xml_diff>
--- a/docker/postgres/users-seed/users-seed.xlsx
+++ b/docker/postgres/users-seed/users-seed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edinson\Documents\SpringBoot\ALBRUGROUP\docker\postgres\users-seed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AC1D63-BD2D-417F-BF50-EEEECD053A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D27726E-5CBB-4490-8610-0E6351E9BB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19500" yWindow="2535" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="1099">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="1105">
   <si>
     <t>empleado_id</t>
   </si>
@@ -3306,9 +3306,6 @@
     <t>WIN</t>
   </si>
   <si>
-    <t>Columna1</t>
-  </si>
-  <si>
     <t>CLARO</t>
   </si>
   <si>
@@ -3322,13 +3319,34 @@
   </si>
   <si>
     <t>jrZY4H4Kr&amp;</t>
+  </si>
+  <si>
+    <t>8zL8B4Fg@A</t>
+  </si>
+  <si>
+    <t>cuMRYVzhig</t>
+  </si>
+  <si>
+    <t>Proveedor</t>
+  </si>
+  <si>
+    <t>AJ_s9h6@#&amp;</t>
+  </si>
+  <si>
+    <t>rLs8TRU4DK</t>
+  </si>
+  <si>
+    <t>FdvCz_mWEo</t>
+  </si>
+  <si>
+    <t>necUE__gxn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3341,14 +3359,6 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -3388,18 +3398,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3420,14 +3428,12 @@
   <autoFilter ref="A1:U76" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="6">
       <filters>
-        <filter val="ASESOR_GTR"/>
         <filter val="ASESOR_VENTAS"/>
-        <filter val="COMMUNITY"/>
       </filters>
     </filterColumn>
     <filterColumn colId="15">
       <filters>
-        <filter val="00:00"/>
+        <filter val="08:00"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3452,7 +3458,7 @@
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="inicio_almuerzo"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="fin_almuerzo"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="PASSWORD"/>
-    <tableColumn id="21" xr3:uid="{23245F2B-70CC-499A-8CBD-C073FFCE2337}" name="Columna1"/>
+    <tableColumn id="21" xr3:uid="{23245F2B-70CC-499A-8CBD-C073FFCE2337}" name="Proveedor"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3747,19 +3753,20 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="12" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="32" customWidth="1"/>
     <col min="11" max="11" width="18" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="16" hidden="1" customWidth="1"/>
     <col min="13" max="14" width="18" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="26" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="14" customWidth="1"/>
+    <col min="16" max="17" width="7.140625" customWidth="1"/>
     <col min="18" max="19" width="18" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="18" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
@@ -3824,7 +3831,7 @@
         <v>19</v>
       </c>
       <c r="U1" t="s">
-        <v>1093</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="2" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -4835,7 +4842,7 @@
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>283</v>
       </c>
@@ -4890,7 +4897,7 @@
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
       <c r="T20" s="2" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -4947,7 +4954,9 @@
       </c>
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
-      <c r="T21" s="2"/>
+      <c r="T21" s="2" t="s">
+        <v>1098</v>
+      </c>
     </row>
     <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
@@ -5341,7 +5350,7 @@
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>412</v>
       </c>
@@ -5396,13 +5405,13 @@
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
       <c r="T29" s="2" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="U29" t="s">
         <v>1092</v>
       </c>
     </row>
-    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>427</v>
       </c>
@@ -6018,7 +6027,7 @@
       <c r="S40" s="2"/>
       <c r="T40" s="2"/>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>584</v>
       </c>
@@ -6133,7 +6142,9 @@
       </c>
       <c r="R42" s="2"/>
       <c r="S42" s="2"/>
-      <c r="T42" s="2"/>
+      <c r="T42" s="2" t="s">
+        <v>1099</v>
+      </c>
     </row>
     <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
@@ -7031,7 +7042,7 @@
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>840</v>
       </c>
@@ -7087,7 +7098,7 @@
       <c r="S59" s="2"/>
       <c r="T59" s="2"/>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>854</v>
       </c>
@@ -7142,13 +7153,13 @@
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
       <c r="T60" s="2" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="U60" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
-    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>868</v>
       </c>
@@ -7202,9 +7213,14 @@
       </c>
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
-      <c r="T61" s="2"/>
+      <c r="T61" s="2" t="s">
+        <v>1104</v>
+      </c>
+      <c r="U61" t="s">
+        <v>1093</v>
+      </c>
     </row>
-    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>882</v>
       </c>
@@ -7258,7 +7274,9 @@
       </c>
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
-      <c r="T62" s="2"/>
+      <c r="T62" s="2" t="s">
+        <v>1101</v>
+      </c>
     </row>
     <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
@@ -7708,7 +7726,7 @@
       <c r="S70" s="2"/>
       <c r="T70" s="2"/>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>1008</v>
       </c>
@@ -7763,13 +7781,13 @@
       <c r="R71" s="2"/>
       <c r="S71" s="2"/>
       <c r="T71" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="U71" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>1022</v>
       </c>
@@ -7879,7 +7897,9 @@
       </c>
       <c r="R73" s="2"/>
       <c r="S73" s="2"/>
-      <c r="T73" s="2"/>
+      <c r="T73" s="2" t="s">
+        <v>1102</v>
+      </c>
     </row>
     <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
@@ -7935,7 +7955,12 @@
       </c>
       <c r="R74" s="2"/>
       <c r="S74" s="2"/>
-      <c r="T74" s="2"/>
+      <c r="T74" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="U74" t="s">
+        <v>1093</v>
+      </c>
     </row>
     <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
@@ -8050,18 +8075,9 @@
       <c r="T76" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="J20" r:id="rId1" xr:uid="{389034BE-AF4B-4311-ABC3-F5C39CB87BDD}"/>
-    <hyperlink ref="J41" r:id="rId2" xr:uid="{2369C96A-5028-4795-89F2-AF6BD153460C}"/>
-    <hyperlink ref="J71" r:id="rId3" xr:uid="{6427C665-EC69-4A12-A2B7-282B8ACD4BC9}"/>
-    <hyperlink ref="I71" r:id="rId4" xr:uid="{128205EE-DCF9-430B-A043-7FAC899FF364}"/>
-    <hyperlink ref="J72" r:id="rId5" xr:uid="{A1E26743-5011-48C7-9992-3DA0C51F1AA3}"/>
-    <hyperlink ref="J60" r:id="rId6" xr:uid="{320CCF57-66E8-46E5-9013-F33B2A1257FA}"/>
-    <hyperlink ref="I60" r:id="rId7" xr:uid="{C4FDBEBF-A328-479F-84F0-1AB8F2459BEE}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: Ships de Oportunidades Mejorado
</commit_message>
<xml_diff>
--- a/docker/postgres/users-seed/users-seed.xlsx
+++ b/docker/postgres/users-seed/users-seed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edinson\Documents\SpringBoot\ALBRUGROUP\docker\postgres\users-seed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D27726E-5CBB-4490-8610-0E6351E9BB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{673A41A6-01CE-4510-AC34-0E6255C5D7E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19500" yWindow="2535" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3428,12 +3428,12 @@
   <autoFilter ref="A1:U76" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="6">
       <filters>
-        <filter val="ASESOR_VENTAS"/>
+        <filter val="COMMUNITY"/>
       </filters>
     </filterColumn>
     <filterColumn colId="15">
       <filters>
-        <filter val="08:00"/>
+        <filter val="15:59"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -4958,7 +4958,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>312</v>
       </c>
@@ -5411,7 +5411,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>427</v>
       </c>
@@ -7159,7 +7159,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>868</v>
       </c>
@@ -7220,7 +7220,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>882</v>
       </c>

</xml_diff>

<commit_message>
Update: Groups de Teams
</commit_message>
<xml_diff>
--- a/docker/postgres/users-seed/users-seed.xlsx
+++ b/docker/postgres/users-seed/users-seed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edinson\Documents\SpringBoot\ALBRUGROUP\docker\postgres\users-seed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{673A41A6-01CE-4510-AC34-0E6255C5D7E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A1526D-6A13-4C88-B5E4-7D5F4B1EDAC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19500" yWindow="2535" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20775" yWindow="5310" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="users-seed" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="1105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="1103">
   <si>
     <t>empleado_id</t>
   </si>
@@ -3321,25 +3321,19 @@
     <t>jrZY4H4Kr&amp;</t>
   </si>
   <si>
-    <t>8zL8B4Fg@A</t>
-  </si>
-  <si>
-    <t>cuMRYVzhig</t>
-  </si>
-  <si>
     <t>Proveedor</t>
   </si>
   <si>
-    <t>AJ_s9h6@#&amp;</t>
-  </si>
-  <si>
-    <t>rLs8TRU4DK</t>
-  </si>
-  <si>
-    <t>FdvCz_mWEo</t>
-  </si>
-  <si>
-    <t>necUE__gxn</t>
+    <t>D#SZoPcZ_Y</t>
+  </si>
+  <si>
+    <t>RLY3Z9Qf3M</t>
+  </si>
+  <si>
+    <t>P5RAVT75A*</t>
+  </si>
+  <si>
+    <t>zVr@ZSCzCd</t>
   </si>
 </sst>
 </file>
@@ -3401,11 +3395,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3428,15 +3424,18 @@
   <autoFilter ref="A1:U76" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="6">
       <filters>
-        <filter val="COMMUNITY"/>
+        <filter val="RRHH"/>
       </filters>
     </filterColumn>
     <filterColumn colId="15">
       <filters>
-        <filter val="15:59"/>
+        <filter val="08:00"/>
       </filters>
     </filterColumn>
   </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A29:U74">
+    <sortCondition ref="G1:G76"/>
+  </sortState>
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="empleado_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="usuario_id"/>
@@ -3831,7 +3830,7 @@
         <v>19</v>
       </c>
       <c r="U1" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="2" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -4058,7 +4057,7 @@
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
     </row>
-    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>83</v>
       </c>
@@ -4112,7 +4111,9 @@
       </c>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
+      <c r="T6" s="2" t="s">
+        <v>1099</v>
+      </c>
     </row>
     <row r="7" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -4955,10 +4956,10 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
       <c r="T21" s="2" t="s">
-        <v>1098</v>
+        <v>1100</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>312</v>
       </c>
@@ -5352,49 +5353,49 @@
     </row>
     <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>412</v>
+        <v>584</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>413</v>
+        <v>585</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>414</v>
+        <v>586</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>415</v>
+        <v>587</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>416</v>
+        <v>588</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>417</v>
+        <v>589</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>418</v>
+        <v>590</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>419</v>
+        <v>591</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>421</v>
+        <v>592</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>593</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>422</v>
+        <v>594</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>423</v>
+        <v>595</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>424</v>
+        <v>596</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>425</v>
+        <v>597</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>426</v>
+        <v>598</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>35</v>
@@ -5405,7 +5406,7 @@
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
       <c r="T29" s="2" t="s">
-        <v>1094</v>
+        <v>1091</v>
       </c>
       <c r="U29" t="s">
         <v>1092</v>
@@ -5413,49 +5414,49 @@
     </row>
     <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>427</v>
+        <v>599</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>428</v>
+        <v>600</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>429</v>
+        <v>601</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>430</v>
+        <v>602</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>431</v>
+        <v>603</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>432</v>
+        <v>604</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>418</v>
+        <v>590</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>433</v>
+        <v>605</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>434</v>
+        <v>606</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>435</v>
+        <v>607</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>436</v>
+        <v>608</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>437</v>
+        <v>609</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>438</v>
+        <v>610</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>439</v>
+        <v>611</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>440</v>
+        <v>612</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>36</v>
@@ -5465,7 +5466,12 @@
       </c>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
+      <c r="T30" s="2" t="s">
+        <v>1101</v>
+      </c>
+      <c r="U30" t="s">
+        <v>1093</v>
+      </c>
     </row>
     <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
@@ -6029,49 +6035,49 @@
     </row>
     <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>584</v>
+        <v>1008</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>585</v>
+        <v>1009</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>586</v>
+        <v>1010</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>587</v>
+        <v>1011</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>588</v>
+        <v>1012</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>589</v>
+        <v>1013</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>590</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>592</v>
+        <v>1014</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>1015</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>593</v>
+        <v>1016</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>594</v>
+        <v>1017</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>595</v>
+        <v>1018</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>596</v>
+        <v>1019</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>597</v>
+        <v>1020</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>598</v>
+        <v>1021</v>
       </c>
       <c r="P41" s="2" t="s">
         <v>35</v>
@@ -6082,69 +6088,67 @@
       <c r="R41" s="2"/>
       <c r="S41" s="2"/>
       <c r="T41" s="2" t="s">
-        <v>1091</v>
+        <v>1096</v>
       </c>
       <c r="U41" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>599</v>
+        <v>1022</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>600</v>
+        <v>1023</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>601</v>
+        <v>1024</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>602</v>
+        <v>1025</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>603</v>
+        <v>1026</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>604</v>
+        <v>1027</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>590</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>605</v>
+        <v>1028</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>607</v>
+        <v>1029</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>1030</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>608</v>
+        <v>1031</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>609</v>
+        <v>1032</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>610</v>
+        <v>1033</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>611</v>
+        <v>1034</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>612</v>
+        <v>1035</v>
       </c>
       <c r="P42" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q42" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="Q42" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="R42" s="2"/>
       <c r="S42" s="2"/>
-      <c r="T42" s="2" t="s">
-        <v>1099</v>
-      </c>
+      <c r="T42" s="2"/>
     </row>
     <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
@@ -7044,55 +7048,55 @@
     </row>
     <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>840</v>
+        <v>1036</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>841</v>
+        <v>1037</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>842</v>
+        <v>1038</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>843</v>
+        <v>1039</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>844</v>
+        <v>1040</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>845</v>
+        <v>1041</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>418</v>
+        <v>590</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>846</v>
+        <v>1042</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>847</v>
+        <v>1043</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>848</v>
+        <v>1044</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>849</v>
+        <v>1045</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>850</v>
+        <v>1046</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>851</v>
+        <v>1047</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>852</v>
+        <v>1048</v>
       </c>
       <c r="O59" s="2" t="s">
-        <v>853</v>
+        <v>1049</v>
       </c>
       <c r="P59" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q59" s="2" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
@@ -7100,171 +7104,166 @@
     </row>
     <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>854</v>
+        <v>1050</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>855</v>
+        <v>1051</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>856</v>
+        <v>1052</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>857</v>
+        <v>1053</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>858</v>
+        <v>1054</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>859</v>
+        <v>417</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>418</v>
+        <v>590</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>860</v>
-      </c>
-      <c r="I60" s="3" t="s">
-        <v>861</v>
-      </c>
-      <c r="J60" s="3" t="s">
-        <v>862</v>
+        <v>1055</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>1056</v>
+      </c>
+      <c r="J60" s="5" t="s">
+        <v>1057</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>863</v>
+        <v>1058</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>864</v>
+        <v>1059</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>865</v>
+        <v>1060</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>866</v>
+        <v>1061</v>
       </c>
       <c r="O60" s="2" t="s">
-        <v>867</v>
+        <v>1062</v>
       </c>
       <c r="P60" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q60" s="2" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
-      <c r="T60" s="2" t="s">
-        <v>1097</v>
-      </c>
-      <c r="U60" t="s">
-        <v>1093</v>
-      </c>
+      <c r="T60" s="2"/>
     </row>
     <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>868</v>
+        <v>412</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>869</v>
+        <v>413</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>870</v>
+        <v>414</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>871</v>
+        <v>415</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>872</v>
+        <v>416</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>873</v>
+        <v>417</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>418</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>874</v>
+        <v>419</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>875</v>
+        <v>420</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>876</v>
+        <v>421</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>877</v>
+        <v>422</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>878</v>
+        <v>423</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>879</v>
+        <v>424</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>880</v>
+        <v>425</v>
       </c>
       <c r="O61" s="2" t="s">
-        <v>881</v>
+        <v>426</v>
       </c>
       <c r="P61" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q61" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="Q61" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
       <c r="T61" s="2" t="s">
-        <v>1104</v>
+        <v>1094</v>
       </c>
       <c r="U61" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>882</v>
+        <v>427</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>883</v>
+        <v>428</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>884</v>
+        <v>429</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>885</v>
+        <v>430</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>886</v>
+        <v>431</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>887</v>
+        <v>432</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>418</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>888</v>
+        <v>433</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>889</v>
+        <v>434</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>890</v>
+        <v>435</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>891</v>
+        <v>436</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>892</v>
+        <v>437</v>
       </c>
       <c r="M62" s="2" t="s">
-        <v>893</v>
+        <v>438</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>894</v>
+        <v>439</v>
       </c>
       <c r="O62" s="2" t="s">
-        <v>895</v>
+        <v>440</v>
       </c>
       <c r="P62" s="2" t="s">
         <v>36</v>
@@ -7275,7 +7274,10 @@
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
       <c r="T62" s="2" t="s">
-        <v>1101</v>
+        <v>1102</v>
+      </c>
+      <c r="U62" t="s">
+        <v>1093</v>
       </c>
     </row>
     <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -7728,49 +7730,49 @@
     </row>
     <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>1008</v>
+        <v>840</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>1009</v>
+        <v>841</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>1010</v>
+        <v>842</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>1011</v>
+        <v>843</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>1012</v>
+        <v>844</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>1013</v>
+        <v>845</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>590</v>
+        <v>418</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>1014</v>
-      </c>
-      <c r="I71" s="3" t="s">
-        <v>1015</v>
-      </c>
-      <c r="J71" s="3" t="s">
-        <v>1016</v>
+        <v>846</v>
+      </c>
+      <c r="I71" s="5" t="s">
+        <v>847</v>
+      </c>
+      <c r="J71" s="5" t="s">
+        <v>848</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>1017</v>
+        <v>849</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>1018</v>
+        <v>850</v>
       </c>
       <c r="M71" s="2" t="s">
-        <v>1019</v>
+        <v>851</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>1020</v>
+        <v>852</v>
       </c>
       <c r="O71" s="2" t="s">
-        <v>1021</v>
+        <v>853</v>
       </c>
       <c r="P71" s="2" t="s">
         <v>35</v>
@@ -7780,58 +7782,53 @@
       </c>
       <c r="R71" s="2"/>
       <c r="S71" s="2"/>
-      <c r="T71" s="2" t="s">
-        <v>1096</v>
-      </c>
-      <c r="U71" t="s">
-        <v>1093</v>
-      </c>
+      <c r="T71" s="2"/>
     </row>
     <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>1022</v>
+        <v>854</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>1023</v>
+        <v>855</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>1024</v>
+        <v>856</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>1025</v>
+        <v>857</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>1026</v>
+        <v>858</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>1027</v>
+        <v>859</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>590</v>
+        <v>418</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>1028</v>
-      </c>
-      <c r="I72" s="2" t="s">
-        <v>1029</v>
+        <v>860</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>861</v>
       </c>
       <c r="J72" s="3" t="s">
-        <v>1030</v>
+        <v>862</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>1031</v>
+        <v>863</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>1032</v>
+        <v>864</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>1033</v>
+        <v>865</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>1034</v>
+        <v>866</v>
       </c>
       <c r="O72" s="2" t="s">
-        <v>1035</v>
+        <v>867</v>
       </c>
       <c r="P72" s="2" t="s">
         <v>35</v>
@@ -7841,53 +7838,58 @@
       </c>
       <c r="R72" s="2"/>
       <c r="S72" s="2"/>
-      <c r="T72" s="2"/>
+      <c r="T72" s="2" t="s">
+        <v>1097</v>
+      </c>
+      <c r="U72" t="s">
+        <v>1093</v>
+      </c>
     </row>
     <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>1036</v>
+        <v>868</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>1037</v>
+        <v>869</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>1038</v>
+        <v>870</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>1039</v>
+        <v>871</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>1040</v>
+        <v>872</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>1041</v>
+        <v>873</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>590</v>
+        <v>418</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>1042</v>
+        <v>874</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>1043</v>
+        <v>875</v>
       </c>
       <c r="J73" s="2" t="s">
-        <v>1044</v>
+        <v>876</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>1045</v>
+        <v>877</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>1046</v>
+        <v>878</v>
       </c>
       <c r="M73" s="2" t="s">
-        <v>1047</v>
+        <v>879</v>
       </c>
       <c r="N73" s="2" t="s">
-        <v>1048</v>
+        <v>880</v>
       </c>
       <c r="O73" s="2" t="s">
-        <v>1049</v>
+        <v>881</v>
       </c>
       <c r="P73" s="2" t="s">
         <v>36</v>
@@ -7897,55 +7899,56 @@
       </c>
       <c r="R73" s="2"/>
       <c r="S73" s="2"/>
-      <c r="T73" s="2" t="s">
-        <v>1102</v>
+      <c r="T73" s="2"/>
+      <c r="U73" t="s">
+        <v>1093</v>
       </c>
     </row>
     <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>1050</v>
+        <v>882</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>1051</v>
+        <v>883</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>1052</v>
+        <v>884</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>1053</v>
+        <v>885</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>1054</v>
+        <v>886</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>417</v>
+        <v>887</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>590</v>
+        <v>418</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>1055</v>
+        <v>888</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>1056</v>
+        <v>889</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>1057</v>
+        <v>890</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>1058</v>
+        <v>891</v>
       </c>
       <c r="L74" s="2" t="s">
-        <v>1059</v>
+        <v>892</v>
       </c>
       <c r="M74" s="2" t="s">
-        <v>1060</v>
+        <v>893</v>
       </c>
       <c r="N74" s="2" t="s">
-        <v>1061</v>
+        <v>894</v>
       </c>
       <c r="O74" s="2" t="s">
-        <v>1062</v>
+        <v>895</v>
       </c>
       <c r="P74" s="2" t="s">
         <v>36</v>
@@ -7955,12 +7958,7 @@
       </c>
       <c r="R74" s="2"/>
       <c r="S74" s="2"/>
-      <c r="T74" s="2" t="s">
-        <v>1103</v>
-      </c>
-      <c r="U74" t="s">
-        <v>1093</v>
-      </c>
+      <c r="T74" s="2"/>
     </row>
     <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">

</xml_diff>

<commit_message>
Update: Leads del Dia 2da propuesta + Fix en responsividad
</commit_message>
<xml_diff>
--- a/docker/postgres/users-seed/users-seed.xlsx
+++ b/docker/postgres/users-seed/users-seed.xlsx
@@ -8,15 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edinson\Documents\SpringBoot\ALBRUGROUP\docker\postgres\users-seed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A1526D-6A13-4C88-B5E4-7D5F4B1EDAC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BDA323-DE96-4FA4-B6AB-F4BE4335CA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20775" yWindow="5310" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10380" yWindow="495" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="users-seed" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="1103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1316" uniqueCount="1105">
   <si>
     <t>empleado_id</t>
   </si>
@@ -3300,9 +3309,6 @@
     <t>00212345000000000075</t>
   </si>
   <si>
-    <t>T$xn539fdY</t>
-  </si>
-  <si>
     <t>WIN</t>
   </si>
   <si>
@@ -3315,9 +3321,6 @@
     <t>o#pkkffwer</t>
   </si>
   <si>
-    <t>vPP-g2LPxp</t>
-  </si>
-  <si>
     <t>jrZY4H4Kr&amp;</t>
   </si>
   <si>
@@ -3330,10 +3333,22 @@
     <t>RLY3Z9Qf3M</t>
   </si>
   <si>
-    <t>P5RAVT75A*</t>
-  </si>
-  <si>
     <t>zVr@ZSCzCd</t>
+  </si>
+  <si>
+    <t>_zDE%JQ8eK</t>
+  </si>
+  <si>
+    <t>Y27WWu-iFM</t>
+  </si>
+  <si>
+    <t>b3wKodwzX@</t>
+  </si>
+  <si>
+    <t>WWSrsk$%@4</t>
+  </si>
+  <si>
+    <t>Gt98*8VQhZ</t>
   </si>
 </sst>
 </file>
@@ -3424,7 +3439,7 @@
   <autoFilter ref="A1:U76" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="6">
       <filters>
-        <filter val="RRHH"/>
+        <filter val="SUPERVISOR_VENTAS"/>
       </filters>
     </filterColumn>
     <filterColumn colId="15">
@@ -3754,7 +3769,7 @@
     <col min="1" max="4" width="12" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5703125" customWidth="1"/>
+    <col min="7" max="7" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="32" customWidth="1"/>
@@ -3830,7 +3845,7 @@
         <v>19</v>
       </c>
       <c r="U1" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="2" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -4057,7 +4072,7 @@
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>83</v>
       </c>
@@ -4112,7 +4127,7 @@
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="7" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -4898,7 +4913,7 @@
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
       <c r="T20" s="2" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -4956,7 +4971,7 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
       <c r="T21" s="2" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -5239,7 +5254,7 @@
       <c r="S26" s="2"/>
       <c r="T26" s="2"/>
     </row>
-    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>384</v>
       </c>
@@ -5293,7 +5308,12 @@
       </c>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
-      <c r="T27" s="2"/>
+      <c r="T27" s="2" t="s">
+        <v>1101</v>
+      </c>
+      <c r="U27" t="s">
+        <v>1091</v>
+      </c>
     </row>
     <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
@@ -5405,12 +5425,7 @@
       </c>
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
-      <c r="T29" s="2" t="s">
-        <v>1091</v>
-      </c>
-      <c r="U29" t="s">
-        <v>1092</v>
-      </c>
+      <c r="T29" s="2"/>
     </row>
     <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
@@ -5467,10 +5482,10 @@
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
       <c r="T30" s="2" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="U30" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -5975,7 +5990,12 @@
       </c>
       <c r="R39" s="2"/>
       <c r="S39" s="2"/>
-      <c r="T39" s="2"/>
+      <c r="T39" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="U39" t="s">
+        <v>1092</v>
+      </c>
     </row>
     <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
@@ -6087,12 +6107,7 @@
       </c>
       <c r="R41" s="2"/>
       <c r="S41" s="2"/>
-      <c r="T41" s="2" t="s">
-        <v>1096</v>
-      </c>
-      <c r="U41" t="s">
-        <v>1093</v>
-      </c>
+      <c r="T41" s="2"/>
     </row>
     <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -6822,7 +6837,7 @@
       <c r="S54" s="2"/>
       <c r="T54" s="2"/>
     </row>
-    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>784</v>
       </c>
@@ -6876,9 +6891,14 @@
       </c>
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
-      <c r="T55" s="2"/>
+      <c r="T55" s="2" t="s">
+        <v>1104</v>
+      </c>
+      <c r="U55" t="s">
+        <v>1092</v>
+      </c>
     </row>
-    <row r="56" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>798</v>
       </c>
@@ -7100,7 +7120,12 @@
       </c>
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
-      <c r="T59" s="2"/>
+      <c r="T59" s="2" t="s">
+        <v>1102</v>
+      </c>
+      <c r="U59" t="s">
+        <v>1092</v>
+      </c>
     </row>
     <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
@@ -7213,10 +7238,10 @@
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
       <c r="T61" s="2" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="U61" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -7274,10 +7299,10 @@
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
       <c r="T62" s="2" t="s">
-        <v>1102</v>
+        <v>1099</v>
       </c>
       <c r="U62" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -7839,10 +7864,10 @@
       <c r="R72" s="2"/>
       <c r="S72" s="2"/>
       <c r="T72" s="2" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="U72" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
@@ -7901,7 +7926,7 @@
       <c r="S73" s="2"/>
       <c r="T73" s="2"/>
       <c r="U73" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update: Ahora se permite ingresar un Gasto del dia anterior y Historicos resuelto diferenciando dia puntual o rango de dias solo indicando el ultimo gasto por dia
</commit_message>
<xml_diff>
--- a/docker/postgres/users-seed/users-seed.xlsx
+++ b/docker/postgres/users-seed/users-seed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edinson\Documents\SpringBoot\ALBRUGROUP\docker\postgres\users-seed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BDA323-DE96-4FA4-B6AB-F4BE4335CA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74862CF0-8CE1-4AEA-A460-2CEA4F56C8AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10380" yWindow="495" windowWidth="16605" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21465" yWindow="12930" windowWidth="16980" windowHeight="5040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="users-seed" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1316" uniqueCount="1105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="1101">
   <si>
     <t>empleado_id</t>
   </si>
@@ -3336,19 +3336,7 @@
     <t>zVr@ZSCzCd</t>
   </si>
   <si>
-    <t>_zDE%JQ8eK</t>
-  </si>
-  <si>
-    <t>Y27WWu-iFM</t>
-  </si>
-  <si>
-    <t>b3wKodwzX@</t>
-  </si>
-  <si>
     <t>WWSrsk$%@4</t>
-  </si>
-  <si>
-    <t>Gt98*8VQhZ</t>
   </si>
 </sst>
 </file>
@@ -3439,6 +3427,7 @@
   <autoFilter ref="A1:U76" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="6">
       <filters>
+        <filter val="ASESOR_GTR"/>
         <filter val="SUPERVISOR_VENTAS"/>
       </filters>
     </filterColumn>
@@ -4690,7 +4679,7 @@
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
     </row>
-    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>240</v>
       </c>
@@ -4746,7 +4735,7 @@
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
     </row>
-    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>255</v>
       </c>
@@ -4802,7 +4791,7 @@
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
     </row>
-    <row r="19" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>269</v>
       </c>
@@ -4858,7 +4847,7 @@
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
     </row>
-    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>283</v>
       </c>
@@ -4916,7 +4905,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>298</v>
       </c>
@@ -4974,7 +4963,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>312</v>
       </c>
@@ -5030,7 +5019,7 @@
       <c r="S22" s="2"/>
       <c r="T22" s="2"/>
     </row>
-    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>326</v>
       </c>
@@ -5086,7 +5075,7 @@
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
     </row>
-    <row r="24" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>341</v>
       </c>
@@ -5142,7 +5131,7 @@
       <c r="S24" s="2"/>
       <c r="T24" s="2"/>
     </row>
-    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>355</v>
       </c>
@@ -5198,7 +5187,7 @@
       <c r="S25" s="2"/>
       <c r="T25" s="2"/>
     </row>
-    <row r="26" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>369</v>
       </c>
@@ -5254,7 +5243,7 @@
       <c r="S26" s="2"/>
       <c r="T26" s="2"/>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>384</v>
       </c>
@@ -5308,14 +5297,9 @@
       </c>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
-      <c r="T27" s="2" t="s">
-        <v>1101</v>
-      </c>
-      <c r="U27" t="s">
-        <v>1091</v>
-      </c>
+      <c r="T27" s="2"/>
     </row>
-    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>398</v>
       </c>
@@ -5371,7 +5355,7 @@
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
     </row>
-    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>584</v>
       </c>
@@ -5427,7 +5411,7 @@
       <c r="S29" s="2"/>
       <c r="T29" s="2"/>
     </row>
-    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>599</v>
       </c>
@@ -5481,14 +5465,9 @@
       </c>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
-      <c r="T30" s="2" t="s">
-        <v>1100</v>
-      </c>
-      <c r="U30" t="s">
-        <v>1091</v>
-      </c>
+      <c r="T30" s="2"/>
     </row>
-    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>441</v>
       </c>
@@ -5544,7 +5523,7 @@
       <c r="S31" s="2"/>
       <c r="T31" s="2"/>
     </row>
-    <row r="32" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>455</v>
       </c>
@@ -5991,7 +5970,7 @@
       <c r="R39" s="2"/>
       <c r="S39" s="2"/>
       <c r="T39" s="2" t="s">
-        <v>1103</v>
+        <v>1100</v>
       </c>
       <c r="U39" t="s">
         <v>1092</v>
@@ -6891,12 +6870,7 @@
       </c>
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
-      <c r="T55" s="2" t="s">
-        <v>1104</v>
-      </c>
-      <c r="U55" t="s">
-        <v>1092</v>
-      </c>
+      <c r="T55" s="2"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
@@ -7066,7 +7040,7 @@
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
     </row>
-    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>1036</v>
       </c>
@@ -7120,14 +7094,9 @@
       </c>
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
-      <c r="T59" s="2" t="s">
-        <v>1102</v>
-      </c>
-      <c r="U59" t="s">
-        <v>1092</v>
-      </c>
+      <c r="T59" s="2"/>
     </row>
-    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>1050</v>
       </c>

</xml_diff>